<commit_message>
WIP Addition & COA Adjsutments
</commit_message>
<xml_diff>
--- a/accountant-skill/data/Jan2026/audit_validation_Jan2026.xlsx
+++ b/accountant-skill/data/Jan2026/audit_validation_Jan2026.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Double-Entry Checks" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross-Module Flow" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Validation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +61,10 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
@@ -117,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -157,10 +162,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -596,11 +604,11 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr"/>
@@ -612,11 +620,11 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
@@ -669,7 +677,7 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -782,7 +790,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Adj accounts=8, TB adj accounts=0</t>
+          <t>Adj accounts=7, TB adj accounts=0</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr"/>
@@ -805,14 +813,14 @@
           <t>Balance Sheet: Assets = Equity + Liabilities</t>
         </is>
       </c>
-      <c r="C23" s="16" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Assets=13,215,750.00, Equity=9,142,750.00, Liabilities=4,073,000.00, Diff=0.00</t>
+          <t>Assets=12,160,750.00, Equity=9,207,750.00, Liabilities=4,073,000.00, Diff=-1,120,000.00</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr"/>
@@ -828,14 +836,14 @@
           <t>Balance Sheet (Dashboard Check)</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Dashboard validation: PASS</t>
+          <t>Dashboard validation: FAIL</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr"/>
@@ -1054,7 +1062,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Adj accounts=8, TB adj accounts=0</t>
+          <t>Adj accounts=7, TB adj accounts=0</t>
         </is>
       </c>
     </row>
@@ -1133,14 +1141,14 @@
           <t>Balance Sheet: Assets = Equity + Liabilities</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Assets=13,215,750.00, Equity=9,142,750.00, Liabilities=4,073,000.00, Diff=0.00</t>
+          <t>Assets=12,160,750.00, Equity=9,207,750.00, Liabilities=4,073,000.00, Diff=-1,120,000.00</t>
         </is>
       </c>
     </row>
@@ -1150,14 +1158,14 @@
           <t>Balance Sheet (Dashboard Check)</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Dashboard validation: PASS</t>
+          <t>Dashboard validation: FAIL</t>
         </is>
       </c>
     </row>
@@ -1169,4 +1177,125 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF0000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Exceptions &amp; Warnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Items requiring attention</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Check Name</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Financial Validation</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Balance Sheet: Assets = Equity + Liabilities</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Assets=12,160,750.00, Equity=9,207,750.00, Liabilities=4,073,000.00, Diff=-1,120,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Financial Validation</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Balance Sheet (Dashboard Check)</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Dashboard validation: FAIL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>